<commit_message>
Add Bug sample modification
</commit_message>
<xml_diff>
--- a/Bug Reports/Bug_Report_SauceDemo.xlsx
+++ b/Bug Reports/Bug_Report_SauceDemo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nites\qa-manual-testing-portfolio\Bug Reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB56F02E-5359-4F66-99EB-75E9DFAEEE5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F4E03AF-451F-4BD4-AE46-7D613079BB20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A86762B5-9B2C-48A0-A558-689114784A9E}"/>
   </bookViews>
@@ -190,12 +190,14 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -523,94 +525,94 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I2" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="J2" s="2" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="F3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
-      <c r="I3" s="2" t="s">
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="J3" s="2" t="s">
         <v>18</v>
       </c>
     </row>

</xml_diff>